<commit_message>
Add English contracts import template download and full import modal i18n.
Translate import instructions and controls for EN mode, generate bilingual XLSX templates, and map English enum values during import.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/static/templates/contracts_template.xlsx
+++ b/static/templates/contracts_template.xlsx
@@ -77,6 +77,73 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>اسم العميل (موجود مسبقاً)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>عقد صيانة</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>شهري</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>12000</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>13800</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>دفعة واحدة</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>نشط</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>EL-0001, EL-0002</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>